<commit_message>
Fully functional 1D Row-Block Placement model with visualization
</commit_message>
<xml_diff>
--- a/sample_instances/input_large.xlsx
+++ b/sample_instances/input_large.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Container-filling_v2/sample_instances/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4FA0A4-C283-284E-9B8A-5B22E6769575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="24160" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="118">
   <si>
     <t>Barcode Item</t>
   </si>
@@ -365,30 +374,20 @@
   </si>
   <si>
     <t>Pallet 1.15x0.77x1.16m  12 sets</t>
+  </si>
+  <si>
+    <t>weight</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -483,59 +482,29 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,24 +513,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffe8e8e8"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FFE8E8E8"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office Theme">
       <a:dk1>
@@ -763,7 +793,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -781,7 +811,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -810,7 +840,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -835,7 +865,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -860,7 +890,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -885,7 +915,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -910,7 +940,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -935,7 +965,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -960,7 +990,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -985,7 +1015,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1010,7 +1040,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1023,9 +1053,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -1042,7 +1078,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1060,7 +1096,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1085,7 +1121,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1110,7 +1146,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1135,7 +1171,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1160,7 +1196,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1185,7 +1221,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1210,7 +1246,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1235,7 +1271,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1260,7 +1296,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1285,7 +1321,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1298,9 +1334,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1314,7 +1356,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1332,7 +1374,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1361,7 +1403,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1386,7 +1428,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1411,7 +1453,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1436,7 +1478,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1461,7 +1503,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1486,7 +1528,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1511,7 +1553,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1536,7 +1578,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1561,7 +1603,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1574,57 +1616,64 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W36"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.1719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" hidden="1" width="8.83333" style="1" customWidth="1"/>
-    <col min="4" max="4" width="58.6719" style="1" customWidth="1"/>
-    <col min="5" max="5" hidden="1" width="8.83333" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.3516" style="1" customWidth="1"/>
-    <col min="7" max="10" hidden="1" width="8.83333" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.1719" style="1" customWidth="1"/>
-    <col min="12" max="16" hidden="1" width="8.83333" style="1" customWidth="1"/>
-    <col min="17" max="17" width="22.1719" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.6719" style="1" customWidth="1"/>
-    <col min="19" max="22" hidden="1" width="8.83333" style="1" customWidth="1"/>
-    <col min="23" max="23" width="8.85156" style="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="58.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" style="1" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" style="1" customWidth="1"/>
+    <col min="7" max="10" width="8.83203125" style="1" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="13.1640625" style="1" customWidth="1"/>
+    <col min="12" max="16" width="8.83203125" style="1" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="22.1640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.6640625" style="1" customWidth="1"/>
+    <col min="19" max="22" width="8.83203125" style="1" hidden="1" customWidth="1"/>
+    <col min="23" max="24" width="8.83203125" style="1" customWidth="1"/>
+    <col min="25" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="2">
+    <row r="1" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3"/>
-      <c r="D1" t="s" s="2">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="3"/>
-      <c r="F1" t="s" s="4">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
-      <c r="K1" t="s" s="6">
+      <c r="K1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="L1" s="5"/>
@@ -1632,31 +1681,33 @@
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
       <c r="P1" s="5"/>
-      <c r="Q1" t="s" s="7">
+      <c r="Q1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="R1" t="s" s="6">
+      <c r="R1" s="6" t="s">
         <v>6</v>
       </c>
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
-      <c r="W1" s="8"/>
+      <c r="W1" s="8" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" t="s" s="2">
+    <row r="2" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="9">
         <v>1037504</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" t="s" s="2">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" t="s" s="4">
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="5"/>
@@ -1672,7 +1723,7 @@
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
       <c r="Q2" s="11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R2" s="10">
         <v>12</v>
@@ -1681,93 +1732,97 @@
       <c r="T2" s="5"/>
       <c r="U2" s="5"/>
       <c r="V2" s="5"/>
-      <c r="W2" s="8"/>
+      <c r="W2" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" t="s" s="2">
+    <row r="3" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="9">
         <v>1037505</v>
       </c>
-      <c r="C3" t="s" s="2">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s" s="2">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s" s="12">
+      <c r="E3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s" s="4">
+      <c r="F3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G3" t="s" s="7">
+      <c r="G3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H3" t="s" s="7">
+      <c r="H3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I3" t="s" s="7">
+      <c r="I3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="J3" t="s" s="7">
+      <c r="J3" s="7" t="s">
         <v>18</v>
       </c>
       <c r="K3" s="10">
-        <v>1</v>
-      </c>
-      <c r="L3" t="s" s="7">
+        <v>3</v>
+      </c>
+      <c r="L3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M3" t="s" s="13">
+      <c r="M3" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="N3" t="s" s="7">
+      <c r="N3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="O3" t="s" s="7">
+      <c r="O3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="P3" t="s" s="7">
+      <c r="P3" s="7" t="s">
         <v>23</v>
       </c>
       <c r="Q3" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R3" s="10">
         <v>9</v>
       </c>
       <c r="S3" s="5"/>
-      <c r="T3" t="s" s="7">
+      <c r="T3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="U3" t="s" s="7">
+      <c r="U3" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="V3" t="s" s="13">
+      <c r="V3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="W3" s="8"/>
+      <c r="W3" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" t="s" s="2">
+    <row r="4" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B4" s="9">
         <v>1089543</v>
       </c>
-      <c r="C4" t="s" s="2">
+      <c r="C4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D4" t="s" s="2">
+      <c r="D4" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="3"/>
-      <c r="F4" t="s" s="4">
+      <c r="F4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="G4" t="s" s="7">
+      <c r="G4" s="7" t="s">
         <v>31</v>
       </c>
       <c r="H4" s="11">
@@ -1777,7 +1832,7 @@
         <v>160</v>
       </c>
       <c r="J4" s="11">
-        <v>1.33493081</v>
+        <v>1.3349308099999999</v>
       </c>
       <c r="K4" s="10">
         <v>1</v>
@@ -1785,13 +1840,13 @@
       <c r="L4" s="11">
         <v>0</v>
       </c>
-      <c r="M4" t="s" s="7">
+      <c r="M4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N4" t="s" s="7">
+      <c r="N4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O4" t="s" s="7">
+      <c r="O4" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P4" s="11">
@@ -1803,38 +1858,40 @@
       <c r="R4" s="10">
         <v>0</v>
       </c>
-      <c r="S4" t="s" s="7">
+      <c r="S4" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T4" s="11">
         <v>1684.8</v>
       </c>
       <c r="U4" s="11">
-        <v>4.00479243</v>
+        <v>4.0047924300000002</v>
       </c>
       <c r="V4" s="11">
-        <v>0.0690481453448276</v>
-      </c>
-      <c r="W4" s="8"/>
+        <v>6.9048145344827602E-2</v>
+      </c>
+      <c r="W4" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" t="s" s="2">
+    <row r="5" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B5" s="9">
         <v>1189072</v>
       </c>
-      <c r="C5" t="s" s="2">
+      <c r="C5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s" s="2">
+      <c r="D5" s="2" t="s">
         <v>37</v>
       </c>
       <c r="E5" s="3"/>
-      <c r="F5" t="s" s="4">
+      <c r="F5" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G5" t="s" s="7">
+      <c r="G5" s="7" t="s">
         <v>39</v>
       </c>
       <c r="H5" s="11">
@@ -1844,7 +1901,7 @@
         <v>90</v>
       </c>
       <c r="J5" s="11">
-        <v>0.62810152</v>
+        <v>0.62810151999999997</v>
       </c>
       <c r="K5" s="10">
         <v>8</v>
@@ -1852,13 +1909,13 @@
       <c r="L5" s="11">
         <v>0</v>
       </c>
-      <c r="M5" t="s" s="7">
+      <c r="M5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N5" t="s" s="7">
+      <c r="N5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O5" t="s" s="7">
+      <c r="O5" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P5" s="11">
@@ -1870,38 +1927,40 @@
       <c r="R5" s="10">
         <v>8</v>
       </c>
-      <c r="S5" t="s" s="7">
+      <c r="S5" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T5" s="11">
         <v>2081.52</v>
       </c>
       <c r="U5" s="11">
-        <v>5.65291368</v>
+        <v>5.6529136800000002</v>
       </c>
       <c r="V5" s="11">
-        <v>0.0974640289655172</v>
-      </c>
-      <c r="W5" s="8"/>
+        <v>9.7464028965517202E-2</v>
+      </c>
+      <c r="W5" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" t="s" s="2">
+    <row r="6" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B6" s="9">
         <v>1109141</v>
       </c>
-      <c r="C6" t="s" s="2">
+      <c r="C6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D6" t="s" s="2">
+      <c r="D6" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="F6" t="s" s="4">
+      <c r="F6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G6" t="s" s="7">
+      <c r="G6" s="7" t="s">
         <v>43</v>
       </c>
       <c r="H6" s="11">
@@ -1911,7 +1970,7 @@
         <v>1440</v>
       </c>
       <c r="J6" s="11">
-        <v>1.40101697</v>
+        <v>1.4010169699999999</v>
       </c>
       <c r="K6" s="10">
         <v>5</v>
@@ -1919,13 +1978,13 @@
       <c r="L6" s="11">
         <v>0</v>
       </c>
-      <c r="M6" t="s" s="7">
+      <c r="M6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N6" t="s" s="7">
+      <c r="N6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O6" t="s" s="7">
+      <c r="O6" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P6" s="11">
@@ -1937,7 +1996,7 @@
       <c r="R6" s="10">
         <v>5</v>
       </c>
-      <c r="S6" t="s" s="7">
+      <c r="S6" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T6" s="11">
@@ -1949,26 +2008,28 @@
       <c r="V6" s="11">
         <v>0</v>
       </c>
-      <c r="W6" s="8"/>
+      <c r="W6" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" t="s" s="2">
+    <row r="7" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B7" s="9">
         <v>1189073</v>
       </c>
-      <c r="C7" t="s" s="2">
+      <c r="C7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s" s="2">
+      <c r="D7" s="2" t="s">
         <v>45</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" t="s" s="4">
+      <c r="F7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G7" t="s" s="7">
+      <c r="G7" s="7" t="s">
         <v>46</v>
       </c>
       <c r="H7" s="11">
@@ -1986,17 +2047,17 @@
       <c r="L7" s="11">
         <v>0</v>
       </c>
-      <c r="M7" t="s" s="7">
+      <c r="M7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N7" t="s" s="7">
+      <c r="N7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O7" t="s" s="7">
+      <c r="O7" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P7" s="11">
-        <v>96.90000000000001</v>
+        <v>96.9</v>
       </c>
       <c r="Q7" s="11">
         <v>3</v>
@@ -2004,7 +2065,7 @@
       <c r="R7" s="10">
         <v>24</v>
       </c>
-      <c r="S7" t="s" s="7">
+      <c r="S7" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T7" s="11">
@@ -2014,28 +2075,30 @@
         <v>1.43986155</v>
       </c>
       <c r="V7" s="11">
-        <v>0.024825199137931</v>
-      </c>
-      <c r="W7" s="8"/>
+        <v>2.4825199137930999E-2</v>
+      </c>
+      <c r="W7" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" t="s" s="2">
+    <row r="8" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B8" s="9">
         <v>1052397</v>
       </c>
-      <c r="C8" t="s" s="2">
+      <c r="C8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D8" t="s" s="2">
+      <c r="D8" s="2" t="s">
         <v>48</v>
       </c>
       <c r="E8" s="3"/>
-      <c r="F8" t="s" s="4">
+      <c r="F8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G8" t="s" s="7">
+      <c r="G8" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H8" s="11">
@@ -2045,7 +2108,7 @@
         <v>200</v>
       </c>
       <c r="J8" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="K8" s="10">
         <v>8</v>
@@ -2053,13 +2116,13 @@
       <c r="L8" s="11">
         <v>0</v>
       </c>
-      <c r="M8" t="s" s="7">
+      <c r="M8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N8" t="s" s="7">
+      <c r="N8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O8" t="s" s="7">
+      <c r="O8" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P8" s="11">
@@ -2071,38 +2134,40 @@
       <c r="R8" s="10">
         <v>8</v>
       </c>
-      <c r="S8" t="s" s="7">
+      <c r="S8" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T8" s="11">
         <v>899.3</v>
       </c>
       <c r="U8" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="V8" s="11">
-        <v>0.0236996886206897</v>
-      </c>
-      <c r="W8" s="8"/>
+        <v>2.3699688620689701E-2</v>
+      </c>
+      <c r="W8" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" t="s" s="2">
+    <row r="9" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B9" s="9">
         <v>1089531</v>
       </c>
-      <c r="C9" t="s" s="2">
+      <c r="C9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D9" t="s" s="2">
+      <c r="D9" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E9" s="3"/>
-      <c r="F9" t="s" s="4">
+      <c r="F9" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G9" t="s" s="7">
+      <c r="G9" s="7" t="s">
         <v>46</v>
       </c>
       <c r="H9" s="11">
@@ -2120,17 +2185,17 @@
       <c r="L9" s="11">
         <v>0</v>
       </c>
-      <c r="M9" t="s" s="7">
+      <c r="M9" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N9" t="s" s="7">
+      <c r="N9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O9" t="s" s="7">
+      <c r="O9" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P9" s="11">
-        <v>85.70999999999999</v>
+        <v>85.71</v>
       </c>
       <c r="Q9" s="11">
         <v>1</v>
@@ -2138,38 +2203,40 @@
       <c r="R9" s="10">
         <v>8</v>
       </c>
-      <c r="S9" t="s" s="7">
+      <c r="S9" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T9" s="11">
         <v>2057.04</v>
       </c>
       <c r="U9" s="11">
-        <v>4.31958465</v>
+        <v>4.3195846500000004</v>
       </c>
       <c r="V9" s="11">
-        <v>0.0744755974137931</v>
-      </c>
-      <c r="W9" s="8"/>
+        <v>7.4475597413793101E-2</v>
+      </c>
+      <c r="W9" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" t="s" s="2">
+    <row r="10" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="9">
         <v>1089535</v>
       </c>
-      <c r="C10" t="s" s="2">
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D10" t="s" s="2">
+      <c r="D10" s="2" t="s">
         <v>54</v>
       </c>
       <c r="E10" s="3"/>
-      <c r="F10" t="s" s="4">
+      <c r="F10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G10" t="s" s="7">
+      <c r="G10" s="7" t="s">
         <v>55</v>
       </c>
       <c r="H10" s="11">
@@ -2179,7 +2246,7 @@
         <v>320</v>
       </c>
       <c r="J10" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="K10" s="10">
         <v>8</v>
@@ -2187,13 +2254,13 @@
       <c r="L10" s="11">
         <v>0</v>
       </c>
-      <c r="M10" t="s" s="7">
+      <c r="M10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N10" t="s" s="7">
+      <c r="N10" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O10" t="s" s="7">
+      <c r="O10" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P10" s="11">
@@ -2205,38 +2272,40 @@
       <c r="R10" s="10">
         <v>8</v>
       </c>
-      <c r="S10" t="s" s="7">
+      <c r="S10" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T10" s="11">
-        <v>946.5599999999999</v>
+        <v>946.56</v>
       </c>
       <c r="U10" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="V10" s="11">
-        <v>0.0255227453448276</v>
-      </c>
-      <c r="W10" s="8"/>
+        <v>2.55227453448276E-2</v>
+      </c>
+      <c r="W10" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" t="s" s="2">
+    <row r="11" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B11" s="9">
         <v>1109133</v>
       </c>
-      <c r="C11" t="s" s="2">
+      <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" t="s" s="2">
+      <c r="D11" s="2" t="s">
         <v>57</v>
       </c>
       <c r="E11" s="3"/>
-      <c r="F11" t="s" s="4">
+      <c r="F11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G11" t="s" s="7">
+      <c r="G11" s="7" t="s">
         <v>55</v>
       </c>
       <c r="H11" s="11">
@@ -2246,7 +2315,7 @@
         <v>320</v>
       </c>
       <c r="J11" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="K11" s="10">
         <v>5</v>
@@ -2254,13 +2323,13 @@
       <c r="L11" s="11">
         <v>0</v>
       </c>
-      <c r="M11" t="s" s="7">
+      <c r="M11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N11" t="s" s="7">
+      <c r="N11" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O11" t="s" s="7">
+      <c r="O11" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P11" s="11">
@@ -2272,38 +2341,40 @@
       <c r="R11" s="10">
         <v>0</v>
       </c>
-      <c r="S11" t="s" s="7">
+      <c r="S11" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T11" s="11">
-        <v>946.5599999999999</v>
+        <v>946.56</v>
       </c>
       <c r="U11" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="V11" s="11">
-        <v>0.0255227453448276</v>
-      </c>
-      <c r="W11" s="8"/>
+        <v>2.55227453448276E-2</v>
+      </c>
+      <c r="W11" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" t="s" s="2">
+    <row r="12" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="9">
         <v>1109140</v>
       </c>
-      <c r="C12" t="s" s="2">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" t="s" s="2">
+      <c r="D12" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E12" s="3"/>
-      <c r="F12" t="s" s="4">
+      <c r="F12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G12" t="s" s="7">
+      <c r="G12" s="7" t="s">
         <v>55</v>
       </c>
       <c r="H12" s="11">
@@ -2313,7 +2384,7 @@
         <v>320</v>
       </c>
       <c r="J12" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="K12" s="10">
         <v>5</v>
@@ -2321,13 +2392,13 @@
       <c r="L12" s="11">
         <v>0</v>
       </c>
-      <c r="M12" t="s" s="7">
+      <c r="M12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N12" t="s" s="7">
+      <c r="N12" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O12" t="s" s="7">
+      <c r="O12" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P12" s="11">
@@ -2339,38 +2410,40 @@
       <c r="R12" s="10">
         <v>5</v>
       </c>
-      <c r="S12" t="s" s="7">
+      <c r="S12" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T12" s="11">
-        <v>946.5599999999999</v>
+        <v>946.56</v>
       </c>
       <c r="U12" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="V12" s="11">
-        <v>0.0255227453448276</v>
-      </c>
-      <c r="W12" s="8"/>
+        <v>2.55227453448276E-2</v>
+      </c>
+      <c r="W12" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" t="s" s="2">
+    <row r="13" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B13" s="9">
         <v>1148370</v>
       </c>
-      <c r="C13" t="s" s="2">
+      <c r="C13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D13" t="s" s="2">
+      <c r="D13" s="2" t="s">
         <v>61</v>
       </c>
       <c r="E13" s="3"/>
-      <c r="F13" t="s" s="4">
+      <c r="F13" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G13" t="s" s="7">
+      <c r="G13" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H13" s="11">
@@ -2380,7 +2453,7 @@
         <v>200</v>
       </c>
       <c r="J13" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="K13" s="10">
         <v>8</v>
@@ -2388,13 +2461,13 @@
       <c r="L13" s="11">
         <v>0</v>
       </c>
-      <c r="M13" t="s" s="7">
+      <c r="M13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N13" t="s" s="7">
+      <c r="N13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O13" t="s" s="7">
+      <c r="O13" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P13" s="11">
@@ -2406,7 +2479,7 @@
       <c r="R13" s="10">
         <v>24</v>
       </c>
-      <c r="S13" t="s" s="7">
+      <c r="S13" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T13" s="11">
@@ -2418,26 +2491,28 @@
       <c r="V13" s="11">
         <v>0</v>
       </c>
-      <c r="W13" s="8"/>
+      <c r="W13" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" t="s" s="2">
+    <row r="14" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B14" s="9">
         <v>1148373</v>
       </c>
-      <c r="C14" t="s" s="2">
+      <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D14" t="s" s="2">
+      <c r="D14" s="2" t="s">
         <v>63</v>
       </c>
       <c r="E14" s="3"/>
-      <c r="F14" t="s" s="4">
+      <c r="F14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G14" t="s" s="7">
+      <c r="G14" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H14" s="11">
@@ -2447,7 +2522,7 @@
         <v>200</v>
       </c>
       <c r="J14" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="K14" s="10">
         <v>5</v>
@@ -2455,13 +2530,13 @@
       <c r="L14" s="11">
         <v>0</v>
       </c>
-      <c r="M14" t="s" s="7">
+      <c r="M14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N14" t="s" s="7">
+      <c r="N14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O14" t="s" s="7">
+      <c r="O14" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P14" s="11">
@@ -2473,38 +2548,40 @@
       <c r="R14" s="10">
         <v>15</v>
       </c>
-      <c r="S14" t="s" s="7">
+      <c r="S14" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T14" s="11">
         <v>835</v>
       </c>
       <c r="U14" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="V14" s="11">
-        <v>0.0236996886206897</v>
-      </c>
-      <c r="W14" s="8"/>
+        <v>2.3699688620689701E-2</v>
+      </c>
+      <c r="W14" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" t="s" s="2">
+    <row r="15" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B15" s="9">
         <v>1148374</v>
       </c>
-      <c r="C15" t="s" s="2">
+      <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D15" t="s" s="2">
+      <c r="D15" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E15" s="3"/>
-      <c r="F15" t="s" s="4">
+      <c r="F15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G15" t="s" s="7">
+      <c r="G15" s="7" t="s">
         <v>55</v>
       </c>
       <c r="H15" s="11">
@@ -2514,7 +2591,7 @@
         <v>320</v>
       </c>
       <c r="J15" s="11">
-        <v>1.48031923</v>
+        <v>1.4803192300000001</v>
       </c>
       <c r="K15" s="10">
         <v>5</v>
@@ -2522,13 +2599,13 @@
       <c r="L15" s="11">
         <v>0</v>
       </c>
-      <c r="M15" t="s" s="7">
+      <c r="M15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N15" t="s" s="7">
+      <c r="N15" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O15" t="s" s="7">
+      <c r="O15" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P15" s="11">
@@ -2540,38 +2617,40 @@
       <c r="R15" s="10">
         <v>5</v>
       </c>
-      <c r="S15" t="s" s="7">
+      <c r="S15" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T15" s="11">
         <v>2480.88</v>
       </c>
       <c r="U15" s="11">
-        <v>4.44095769</v>
+        <v>4.4409576900000003</v>
       </c>
       <c r="V15" s="11">
-        <v>0.0765682360344828</v>
-      </c>
-      <c r="W15" s="8"/>
+        <v>7.6568236034482803E-2</v>
+      </c>
+      <c r="W15" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" t="s" s="2">
+    <row r="16" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B16" s="9">
         <v>1167769</v>
       </c>
-      <c r="C16" t="s" s="2">
+      <c r="C16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D16" t="s" s="2">
+      <c r="D16" s="2" t="s">
         <v>67</v>
       </c>
       <c r="E16" s="3"/>
-      <c r="F16" t="s" s="4">
+      <c r="F16" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G16" t="s" s="7">
+      <c r="G16" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H16" s="11">
@@ -2581,7 +2660,7 @@
         <v>200</v>
       </c>
       <c r="J16" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="K16" s="10">
         <v>8</v>
@@ -2589,13 +2668,13 @@
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" t="s" s="7">
+      <c r="M16" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N16" t="s" s="7">
+      <c r="N16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O16" t="s" s="7">
+      <c r="O16" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P16" s="11">
@@ -2607,38 +2686,40 @@
       <c r="R16" s="10">
         <v>40</v>
       </c>
-      <c r="S16" t="s" s="7">
+      <c r="S16" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T16" s="11">
-        <v>2298.3</v>
+        <v>2298.3000000000002</v>
       </c>
       <c r="U16" s="11">
-        <v>4.12374582</v>
+        <v>4.1237458199999999</v>
       </c>
       <c r="V16" s="11">
-        <v>0.071099065862069</v>
-      </c>
-      <c r="W16" s="8"/>
+        <v>7.1099065862069002E-2</v>
+      </c>
+      <c r="W16" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" t="s" s="2">
+    <row r="17" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B17" s="9">
         <v>1167772</v>
       </c>
-      <c r="C17" t="s" s="2">
+      <c r="C17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D17" t="s" s="2">
+      <c r="D17" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E17" s="3"/>
-      <c r="F17" t="s" s="4">
+      <c r="F17" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G17" t="s" s="7">
+      <c r="G17" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H17" s="11">
@@ -2648,7 +2729,7 @@
         <v>200</v>
       </c>
       <c r="J17" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="K17" s="10">
         <v>4</v>
@@ -2656,13 +2737,13 @@
       <c r="L17" s="11">
         <v>0</v>
       </c>
-      <c r="M17" t="s" s="7">
+      <c r="M17" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N17" t="s" s="7">
+      <c r="N17" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O17" t="s" s="7">
+      <c r="O17" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P17" s="11">
@@ -2674,38 +2755,40 @@
       <c r="R17" s="10">
         <v>20</v>
       </c>
-      <c r="S17" t="s" s="7">
+      <c r="S17" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T17" s="11">
         <v>766.1</v>
       </c>
       <c r="U17" s="11">
-        <v>1.37458194</v>
+        <v>1.3745819399999999</v>
       </c>
       <c r="V17" s="11">
-        <v>0.0236996886206897</v>
-      </c>
-      <c r="W17" s="8"/>
+        <v>2.3699688620689701E-2</v>
+      </c>
+      <c r="W17" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" t="s" s="2">
+    <row r="18" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B18" s="9">
         <v>1188995</v>
       </c>
-      <c r="C18" t="s" s="2">
+      <c r="C18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D18" t="s" s="2">
+      <c r="D18" s="2" t="s">
         <v>73</v>
       </c>
       <c r="E18" s="3"/>
-      <c r="F18" t="s" s="4">
+      <c r="F18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G18" t="s" s="7">
+      <c r="G18" s="7" t="s">
         <v>74</v>
       </c>
       <c r="H18" s="11">
@@ -2723,17 +2806,17 @@
       <c r="L18" s="11">
         <v>0</v>
       </c>
-      <c r="M18" t="s" s="7">
+      <c r="M18" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N18" t="s" s="7">
+      <c r="N18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O18" t="s" s="7">
+      <c r="O18" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P18" s="11">
-        <v>93.26000000000001</v>
+        <v>93.26</v>
       </c>
       <c r="Q18" s="11">
         <v>13</v>
@@ -2741,38 +2824,40 @@
       <c r="R18" s="10">
         <v>39</v>
       </c>
-      <c r="S18" t="s" s="7">
+      <c r="S18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T18" s="11">
         <v>3730.4</v>
       </c>
       <c r="U18" s="11">
-        <v>8.0624436</v>
+        <v>8.0624435999999999</v>
       </c>
       <c r="V18" s="11">
-        <v>0.139007648275862</v>
-      </c>
-      <c r="W18" s="8"/>
+        <v>0.13900764827586201</v>
+      </c>
+      <c r="W18" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" t="s" s="2">
+    <row r="19" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B19" s="9">
         <v>1167770</v>
       </c>
-      <c r="C19" t="s" s="2">
+      <c r="C19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D19" t="s" s="2">
+      <c r="D19" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E19" s="3"/>
-      <c r="F19" t="s" s="4">
+      <c r="F19" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G19" t="s" s="7">
+      <c r="G19" s="7" t="s">
         <v>77</v>
       </c>
       <c r="H19" s="11">
@@ -2782,7 +2867,7 @@
         <v>176</v>
       </c>
       <c r="J19" s="11">
-        <v>1.22919352</v>
+        <v>1.2291935199999999</v>
       </c>
       <c r="K19" s="10">
         <v>8</v>
@@ -2790,13 +2875,13 @@
       <c r="L19" s="11">
         <v>0</v>
       </c>
-      <c r="M19" t="s" s="7">
+      <c r="M19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N19" t="s" s="7">
+      <c r="N19" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O19" t="s" s="7">
+      <c r="O19" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P19" s="11">
@@ -2808,38 +2893,40 @@
       <c r="R19" s="10">
         <v>0</v>
       </c>
-      <c r="S19" t="s" s="7">
+      <c r="S19" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T19" s="11">
-        <v>2273.2</v>
+        <v>2273.1999999999998</v>
       </c>
       <c r="U19" s="11">
-        <v>6.1459676</v>
+        <v>6.1459675999999996</v>
       </c>
       <c r="V19" s="11">
         <v>0.10596495862069</v>
       </c>
-      <c r="W19" s="8"/>
+      <c r="W19" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" t="s" s="2">
+    <row r="20" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B20" s="9">
         <v>1167773</v>
       </c>
-      <c r="C20" t="s" s="2">
+      <c r="C20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D20" t="s" s="2">
+      <c r="D20" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E20" s="3"/>
-      <c r="F20" t="s" s="4">
+      <c r="F20" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G20" t="s" s="7">
+      <c r="G20" s="7" t="s">
         <v>80</v>
       </c>
       <c r="H20" s="11">
@@ -2849,7 +2936,7 @@
         <v>270</v>
       </c>
       <c r="J20" s="11">
-        <v>0.62810152</v>
+        <v>0.62810151999999997</v>
       </c>
       <c r="K20" s="10">
         <v>4</v>
@@ -2857,13 +2944,13 @@
       <c r="L20" s="11">
         <v>0</v>
       </c>
-      <c r="M20" t="s" s="7">
+      <c r="M20" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N20" t="s" s="7">
+      <c r="N20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O20" t="s" s="7">
+      <c r="O20" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P20" s="11">
@@ -2875,38 +2962,40 @@
       <c r="R20" s="10">
         <v>0</v>
       </c>
-      <c r="S20" t="s" s="7">
+      <c r="S20" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T20" s="11">
         <v>3125.46</v>
       </c>
       <c r="U20" s="11">
-        <v>8.165319759999999</v>
+        <v>8.1653197599999991</v>
       </c>
       <c r="V20" s="11">
-        <v>0.140781375172414</v>
-      </c>
-      <c r="W20" s="8"/>
+        <v>0.14078137517241399</v>
+      </c>
+      <c r="W20" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" t="s" s="2">
+    <row r="21" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B21" s="9">
         <v>1188996</v>
       </c>
-      <c r="C21" t="s" s="2">
+      <c r="C21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D21" t="s" s="2">
+      <c r="D21" s="2" t="s">
         <v>82</v>
       </c>
       <c r="E21" s="3"/>
-      <c r="F21" t="s" s="4">
+      <c r="F21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G21" t="s" s="7">
+      <c r="G21" s="7" t="s">
         <v>74</v>
       </c>
       <c r="H21" s="11">
@@ -2924,17 +3013,17 @@
       <c r="L21" s="11">
         <v>0</v>
       </c>
-      <c r="M21" t="s" s="7">
+      <c r="M21" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N21" t="s" s="7">
+      <c r="N21" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O21" t="s" s="7">
+      <c r="O21" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P21" s="11">
-        <v>93.26000000000001</v>
+        <v>93.26</v>
       </c>
       <c r="Q21" s="11">
         <v>0</v>
@@ -2942,7 +3031,7 @@
       <c r="R21" s="10">
         <v>0</v>
       </c>
-      <c r="S21" t="s" s="7">
+      <c r="S21" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T21" s="11">
@@ -2954,26 +3043,28 @@
       <c r="V21" s="11">
         <v>0</v>
       </c>
-      <c r="W21" s="8"/>
+      <c r="W21" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" t="s" s="2">
+    <row r="22" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B22" s="9">
         <v>1188998</v>
       </c>
-      <c r="C22" t="s" s="2">
+      <c r="C22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D22" t="s" s="2">
+      <c r="D22" s="2" t="s">
         <v>84</v>
       </c>
       <c r="E22" s="3"/>
-      <c r="F22" t="s" s="4">
+      <c r="F22" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G22" t="s" s="7">
+      <c r="G22" s="7" t="s">
         <v>77</v>
       </c>
       <c r="H22" s="11">
@@ -2983,7 +3074,7 @@
         <v>176</v>
       </c>
       <c r="J22" s="11">
-        <v>1.22919352</v>
+        <v>1.2291935199999999</v>
       </c>
       <c r="K22" s="10">
         <v>8</v>
@@ -2991,13 +3082,13 @@
       <c r="L22" s="11">
         <v>0</v>
       </c>
-      <c r="M22" t="s" s="7">
+      <c r="M22" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N22" t="s" s="7">
+      <c r="N22" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O22" t="s" s="7">
+      <c r="O22" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P22" s="11">
@@ -3009,7 +3100,7 @@
       <c r="R22" s="10">
         <v>0</v>
       </c>
-      <c r="S22" t="s" s="7">
+      <c r="S22" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T22" s="11">
@@ -3021,26 +3112,28 @@
       <c r="V22" s="11">
         <v>0</v>
       </c>
-      <c r="W22" s="8"/>
+      <c r="W22" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" t="s" s="2">
+    <row r="23" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>85</v>
       </c>
       <c r="B23" s="9">
         <v>1188999</v>
       </c>
-      <c r="C23" t="s" s="2">
+      <c r="C23" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D23" t="s" s="2">
+      <c r="D23" s="2" t="s">
         <v>86</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" t="s" s="4">
+      <c r="F23" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G23" t="s" s="7">
+      <c r="G23" s="7" t="s">
         <v>80</v>
       </c>
       <c r="H23" s="11">
@@ -3050,7 +3143,7 @@
         <v>270</v>
       </c>
       <c r="J23" s="11">
-        <v>0.62810152</v>
+        <v>0.62810151999999997</v>
       </c>
       <c r="K23" s="10">
         <v>4</v>
@@ -3058,13 +3151,13 @@
       <c r="L23" s="11">
         <v>0</v>
       </c>
-      <c r="M23" t="s" s="7">
+      <c r="M23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N23" t="s" s="7">
+      <c r="N23" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O23" t="s" s="7">
+      <c r="O23" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P23" s="11">
@@ -3076,7 +3169,7 @@
       <c r="R23" s="10">
         <v>0</v>
       </c>
-      <c r="S23" t="s" s="7">
+      <c r="S23" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T23" s="11">
@@ -3088,26 +3181,28 @@
       <c r="V23" s="11">
         <v>0</v>
       </c>
-      <c r="W23" s="8"/>
+      <c r="W23" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" t="s" s="2">
+    <row r="24" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B24" s="9">
         <v>1188997</v>
       </c>
-      <c r="C24" t="s" s="2">
+      <c r="C24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D24" t="s" s="2">
+      <c r="D24" s="2" t="s">
         <v>88</v>
       </c>
       <c r="E24" s="3"/>
-      <c r="F24" t="s" s="4">
+      <c r="F24" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G24" t="s" s="7">
+      <c r="G24" s="7" t="s">
         <v>74</v>
       </c>
       <c r="H24" s="11">
@@ -3125,17 +3220,17 @@
       <c r="L24" s="11">
         <v>0</v>
       </c>
-      <c r="M24" t="s" s="7">
+      <c r="M24" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N24" t="s" s="7">
+      <c r="N24" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O24" t="s" s="7">
+      <c r="O24" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P24" s="11">
-        <v>93.26000000000001</v>
+        <v>93.26</v>
       </c>
       <c r="Q24" s="11">
         <v>0</v>
@@ -3143,7 +3238,7 @@
       <c r="R24" s="10">
         <v>0</v>
       </c>
-      <c r="S24" t="s" s="7">
+      <c r="S24" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T24" s="11">
@@ -3155,26 +3250,28 @@
       <c r="V24" s="11">
         <v>0</v>
       </c>
-      <c r="W24" s="8"/>
+      <c r="W24" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" t="s" s="2">
+    <row r="25" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>89</v>
       </c>
       <c r="B25" s="9">
         <v>1189014</v>
       </c>
-      <c r="C25" t="s" s="2">
+      <c r="C25" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D25" t="s" s="2">
+      <c r="D25" s="2" t="s">
         <v>90</v>
       </c>
       <c r="E25" s="3"/>
-      <c r="F25" t="s" s="4">
+      <c r="F25" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G25" t="s" s="7">
+      <c r="G25" s="7" t="s">
         <v>77</v>
       </c>
       <c r="H25" s="11">
@@ -3184,7 +3281,7 @@
         <v>176</v>
       </c>
       <c r="J25" s="11">
-        <v>1.15437398</v>
+        <v>1.1543739799999999</v>
       </c>
       <c r="K25" s="10">
         <v>4</v>
@@ -3192,13 +3289,13 @@
       <c r="L25" s="11">
         <v>0</v>
       </c>
-      <c r="M25" t="s" s="7">
+      <c r="M25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N25" t="s" s="7">
+      <c r="N25" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O25" t="s" s="7">
+      <c r="O25" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P25" s="11">
@@ -3210,7 +3307,7 @@
       <c r="R25" s="10">
         <v>0</v>
       </c>
-      <c r="S25" t="s" s="7">
+      <c r="S25" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T25" s="11">
@@ -3222,26 +3319,28 @@
       <c r="V25" s="11">
         <v>0</v>
       </c>
-      <c r="W25" s="8"/>
+      <c r="W25" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" t="s" s="2">
+    <row r="26" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>92</v>
       </c>
       <c r="B26" s="9">
         <v>1189015</v>
       </c>
-      <c r="C26" t="s" s="2">
+      <c r="C26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D26" t="s" s="2">
+      <c r="D26" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E26" s="3"/>
-      <c r="F26" t="s" s="4">
+      <c r="F26" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G26" t="s" s="7">
+      <c r="G26" s="7" t="s">
         <v>80</v>
       </c>
       <c r="H26" s="11">
@@ -3251,7 +3350,7 @@
         <v>270</v>
       </c>
       <c r="J26" s="11">
-        <v>0.62810152</v>
+        <v>0.62810151999999997</v>
       </c>
       <c r="K26" s="10">
         <v>4</v>
@@ -3259,13 +3358,13 @@
       <c r="L26" s="11">
         <v>0</v>
       </c>
-      <c r="M26" t="s" s="7">
+      <c r="M26" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N26" t="s" s="7">
+      <c r="N26" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O26" t="s" s="7">
+      <c r="O26" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P26" s="11">
@@ -3277,7 +3376,7 @@
       <c r="R26" s="10">
         <v>0</v>
       </c>
-      <c r="S26" t="s" s="7">
+      <c r="S26" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T26" s="11">
@@ -3289,26 +3388,28 @@
       <c r="V26" s="11">
         <v>0</v>
       </c>
-      <c r="W26" s="8"/>
+      <c r="W26" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" t="s" s="2">
+    <row r="27" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>94</v>
       </c>
       <c r="B27" s="9">
         <v>1189016</v>
       </c>
-      <c r="C27" t="s" s="2">
+      <c r="C27" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D27" t="s" s="2">
+      <c r="D27" s="2" t="s">
         <v>95</v>
       </c>
       <c r="E27" s="3"/>
-      <c r="F27" t="s" s="4">
+      <c r="F27" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G27" t="s" s="7">
+      <c r="G27" s="7" t="s">
         <v>96</v>
       </c>
       <c r="H27" s="11">
@@ -3318,7 +3419,7 @@
         <v>352</v>
       </c>
       <c r="J27" s="11">
-        <v>0.78199409</v>
+        <v>0.78199408999999998</v>
       </c>
       <c r="K27" s="10">
         <v>4</v>
@@ -3326,13 +3427,13 @@
       <c r="L27" s="11">
         <v>0</v>
       </c>
-      <c r="M27" t="s" s="7">
+      <c r="M27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N27" t="s" s="7">
+      <c r="N27" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O27" t="s" s="7">
+      <c r="O27" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P27" s="11">
@@ -3344,7 +3445,7 @@
       <c r="R27" s="10">
         <v>0</v>
       </c>
-      <c r="S27" t="s" s="7">
+      <c r="S27" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T27" s="11">
@@ -3356,26 +3457,28 @@
       <c r="V27" s="11">
         <v>0</v>
       </c>
-      <c r="W27" s="8"/>
+      <c r="W27" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" t="s" s="2">
+    <row r="28" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B28" s="9">
         <v>1189025</v>
       </c>
-      <c r="C28" t="s" s="2">
+      <c r="C28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D28" t="s" s="2">
+      <c r="D28" s="2" t="s">
         <v>98</v>
       </c>
       <c r="E28" s="3"/>
-      <c r="F28" t="s" s="4">
+      <c r="F28" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G28" t="s" s="7">
+      <c r="G28" s="7" t="s">
         <v>96</v>
       </c>
       <c r="H28" s="11">
@@ -3385,7 +3488,7 @@
         <v>352</v>
       </c>
       <c r="J28" s="11">
-        <v>0.78199409</v>
+        <v>0.78199408999999998</v>
       </c>
       <c r="K28" s="10">
         <v>8</v>
@@ -3393,13 +3496,13 @@
       <c r="L28" s="11">
         <v>0</v>
       </c>
-      <c r="M28" t="s" s="7">
+      <c r="M28" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N28" t="s" s="7">
+      <c r="N28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O28" t="s" s="7">
+      <c r="O28" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P28" s="11">
@@ -3411,7 +3514,7 @@
       <c r="R28" s="10">
         <v>0</v>
       </c>
-      <c r="S28" t="s" s="7">
+      <c r="S28" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T28" s="11">
@@ -3423,26 +3526,28 @@
       <c r="V28" s="11">
         <v>0</v>
       </c>
-      <c r="W28" s="8"/>
+      <c r="W28" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" t="s" s="2">
+    <row r="29" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>99</v>
       </c>
       <c r="B29" s="9">
         <v>1189026</v>
       </c>
-      <c r="C29" t="s" s="2">
+      <c r="C29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D29" t="s" s="2">
+      <c r="D29" s="2" t="s">
         <v>100</v>
       </c>
       <c r="E29" s="3"/>
-      <c r="F29" t="s" s="4">
+      <c r="F29" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="G29" t="s" s="7">
+      <c r="G29" s="7" t="s">
         <v>96</v>
       </c>
       <c r="H29" s="11">
@@ -3452,7 +3557,7 @@
         <v>352</v>
       </c>
       <c r="J29" s="11">
-        <v>0.78199409</v>
+        <v>0.78199408999999998</v>
       </c>
       <c r="K29" s="10">
         <v>4</v>
@@ -3460,13 +3565,13 @@
       <c r="L29" s="11">
         <v>0</v>
       </c>
-      <c r="M29" t="s" s="7">
+      <c r="M29" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N29" t="s" s="7">
+      <c r="N29" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O29" t="s" s="7">
+      <c r="O29" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P29" s="11">
@@ -3478,7 +3583,7 @@
       <c r="R29" s="10">
         <v>0</v>
       </c>
-      <c r="S29" t="s" s="7">
+      <c r="S29" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T29" s="11">
@@ -3490,26 +3595,28 @@
       <c r="V29" s="11">
         <v>0</v>
       </c>
-      <c r="W29" s="8"/>
+      <c r="W29" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" t="s" s="2">
+    <row r="30" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B30" s="9">
         <v>1189024</v>
       </c>
-      <c r="C30" t="s" s="2">
+      <c r="C30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D30" t="s" s="2">
+      <c r="D30" s="2" t="s">
         <v>103</v>
       </c>
       <c r="E30" s="3"/>
-      <c r="F30" t="s" s="4">
+      <c r="F30" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G30" t="s" s="7">
+      <c r="G30" s="7" t="s">
         <v>74</v>
       </c>
       <c r="H30" s="11">
@@ -3527,13 +3634,13 @@
       <c r="L30" s="11">
         <v>0</v>
       </c>
-      <c r="M30" t="s" s="7">
+      <c r="M30" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N30" t="s" s="7">
+      <c r="N30" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O30" t="s" s="7">
+      <c r="O30" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P30" s="11">
@@ -3545,7 +3652,7 @@
       <c r="R30" s="10">
         <v>0</v>
       </c>
-      <c r="S30" t="s" s="7">
+      <c r="S30" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T30" s="11">
@@ -3557,26 +3664,28 @@
       <c r="V30" s="11">
         <v>0</v>
       </c>
-      <c r="W30" s="8"/>
+      <c r="W30" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" t="s" s="2">
+    <row r="31" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B31" s="9">
         <v>1189027</v>
       </c>
-      <c r="C31" t="s" s="2">
+      <c r="C31" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D31" t="s" s="2">
+      <c r="D31" s="2" t="s">
         <v>105</v>
       </c>
       <c r="E31" s="3"/>
-      <c r="F31" t="s" s="4">
+      <c r="F31" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="G31" t="s" s="7">
+      <c r="G31" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H31" s="11">
@@ -3586,7 +3695,7 @@
         <v>176</v>
       </c>
       <c r="J31" s="11">
-        <v>1.15437398</v>
+        <v>1.1543739799999999</v>
       </c>
       <c r="K31" s="10">
         <v>5</v>
@@ -3594,25 +3703,25 @@
       <c r="L31" s="11">
         <v>0</v>
       </c>
-      <c r="M31" t="s" s="7">
+      <c r="M31" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N31" t="s" s="7">
+      <c r="N31" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O31" t="s" s="7">
+      <c r="O31" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P31" s="11">
         <v>119.34</v>
       </c>
       <c r="Q31" s="11">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R31" s="10">
         <v>0</v>
       </c>
-      <c r="S31" t="s" s="7">
+      <c r="S31" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T31" s="11">
@@ -3624,26 +3733,28 @@
       <c r="V31" s="11">
         <v>0</v>
       </c>
-      <c r="W31" s="8"/>
+      <c r="W31" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" t="s" s="2">
+    <row r="32" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>108</v>
       </c>
       <c r="B32" s="9">
         <v>1189029</v>
       </c>
-      <c r="C32" t="s" s="2">
+      <c r="C32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D32" t="s" s="2">
+      <c r="D32" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E32" s="3"/>
-      <c r="F32" t="s" s="4">
+      <c r="F32" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="G32" t="s" s="7">
+      <c r="G32" s="7" t="s">
         <v>80</v>
       </c>
       <c r="H32" s="11">
@@ -3653,7 +3764,7 @@
         <v>270</v>
       </c>
       <c r="J32" s="11">
-        <v>0.62810152</v>
+        <v>0.62810151999999997</v>
       </c>
       <c r="K32" s="10">
         <v>5</v>
@@ -3661,17 +3772,17 @@
       <c r="L32" s="11">
         <v>0</v>
       </c>
-      <c r="M32" t="s" s="7">
+      <c r="M32" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N32" t="s" s="7">
+      <c r="N32" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O32" t="s" s="7">
+      <c r="O32" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P32" s="11">
-        <v>84.15000000000001</v>
+        <v>84.15</v>
       </c>
       <c r="Q32" s="11">
         <v>2</v>
@@ -3679,7 +3790,7 @@
       <c r="R32" s="10">
         <v>10</v>
       </c>
-      <c r="S32" t="s" s="7">
+      <c r="S32" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T32" s="11">
@@ -3691,26 +3802,28 @@
       <c r="V32" s="11">
         <v>0</v>
       </c>
-      <c r="W32" s="8"/>
+      <c r="W32" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" t="s" s="2">
+    <row r="33" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>110</v>
       </c>
       <c r="B33" s="9">
         <v>1189028</v>
       </c>
-      <c r="C33" t="s" s="2">
+      <c r="C33" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D33" t="s" s="2">
+      <c r="D33" s="2" t="s">
         <v>111</v>
       </c>
       <c r="E33" s="3"/>
-      <c r="F33" t="s" s="4">
+      <c r="F33" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="G33" t="s" s="7">
+      <c r="G33" s="7" t="s">
         <v>112</v>
       </c>
       <c r="H33" s="11">
@@ -3720,7 +3833,7 @@
         <v>400</v>
       </c>
       <c r="J33" s="11">
-        <v>0.80624436</v>
+        <v>0.80624435999999999</v>
       </c>
       <c r="K33" s="10">
         <v>5</v>
@@ -3728,13 +3841,13 @@
       <c r="L33" s="11">
         <v>0</v>
       </c>
-      <c r="M33" t="s" s="7">
+      <c r="M33" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N33" t="s" s="7">
+      <c r="N33" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O33" t="s" s="7">
+      <c r="O33" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P33" s="11">
@@ -3746,7 +3859,7 @@
       <c r="R33" s="10">
         <v>5</v>
       </c>
-      <c r="S33" t="s" s="7">
+      <c r="S33" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T33" s="11">
@@ -3758,26 +3871,28 @@
       <c r="V33" s="11">
         <v>0</v>
       </c>
-      <c r="W33" s="8"/>
+      <c r="W33" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" t="s" s="2">
+    <row r="34" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>113</v>
       </c>
       <c r="B34" s="9">
         <v>1189040</v>
       </c>
-      <c r="C34" t="s" s="2">
+      <c r="C34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D34" t="s" s="2">
+      <c r="D34" s="2" t="s">
         <v>114</v>
       </c>
       <c r="E34" s="3"/>
-      <c r="F34" t="s" s="4">
+      <c r="F34" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="G34" t="s" s="7">
+      <c r="G34" s="7" t="s">
         <v>112</v>
       </c>
       <c r="H34" s="11">
@@ -3787,7 +3902,7 @@
         <v>400</v>
       </c>
       <c r="J34" s="11">
-        <v>0.80624436</v>
+        <v>0.80624435999999999</v>
       </c>
       <c r="K34" s="14">
         <v>1</v>
@@ -3795,13 +3910,13 @@
       <c r="L34" s="11">
         <v>0</v>
       </c>
-      <c r="M34" t="s" s="7">
+      <c r="M34" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N34" t="s" s="7">
+      <c r="N34" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O34" t="s" s="7">
+      <c r="O34" s="7" t="s">
         <v>34</v>
       </c>
       <c r="P34" s="11">
@@ -3813,7 +3928,7 @@
       <c r="R34" s="14">
         <v>0</v>
       </c>
-      <c r="S34" t="s" s="7">
+      <c r="S34" s="7" t="s">
         <v>35</v>
       </c>
       <c r="T34" s="11">
@@ -3823,20 +3938,22 @@
         <v>1.61248872</v>
       </c>
       <c r="V34" s="11">
-        <v>0.0278015296551724</v>
-      </c>
-      <c r="W34" s="8"/>
+        <v>2.7801529655172401E-2</v>
+      </c>
+      <c r="W34" s="8">
+        <v>100</v>
+      </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
+    <row r="35" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
-      <c r="C35" t="s" s="2">
+      <c r="C35" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
-      <c r="G35" t="s" s="2">
+      <c r="G35" s="2" t="s">
         <v>112</v>
       </c>
       <c r="H35" s="9">
@@ -3846,50 +3963,50 @@
         <v>400</v>
       </c>
       <c r="J35" s="9">
-        <v>0.80624436</v>
+        <v>0.80624435999999999</v>
       </c>
       <c r="K35" s="15"/>
       <c r="L35" s="9">
         <v>0</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="M35" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N35" t="s" s="2">
+      <c r="N35" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O35" t="s" s="2">
+      <c r="O35" s="2" t="s">
         <v>34</v>
       </c>
       <c r="P35" s="9">
-        <v>69.34999999999999</v>
+        <v>69.349999999999994</v>
       </c>
       <c r="Q35" s="3"/>
       <c r="R35" s="15"/>
-      <c r="S35" t="s" s="2">
+      <c r="S35" s="2" t="s">
         <v>35</v>
       </c>
       <c r="T35" s="9">
         <v>346.75</v>
       </c>
       <c r="U35" s="9">
-        <v>0.80624436</v>
+        <v>0.80624435999999999</v>
       </c>
       <c r="V35" s="9">
-        <v>0.0139007648275862</v>
+        <v>1.39007648275862E-2</v>
       </c>
       <c r="W35" s="3"/>
     </row>
-    <row r="36" ht="16" customHeight="1">
+    <row r="36" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
-      <c r="C36" t="s" s="2">
+      <c r="C36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
-      <c r="G36" t="s" s="2">
+      <c r="G36" s="2" t="s">
         <v>116</v>
       </c>
       <c r="H36" s="9">
@@ -3905,13 +4022,13 @@
       <c r="L36" s="9">
         <v>0</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="M36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N36" t="s" s="2">
+      <c r="N36" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O36" t="s" s="2">
+      <c r="O36" s="2" t="s">
         <v>34</v>
       </c>
       <c r="P36" s="9">
@@ -3919,7 +4036,7 @@
       </c>
       <c r="Q36" s="3"/>
       <c r="R36" s="15"/>
-      <c r="S36" t="s" s="2">
+      <c r="S36" s="2" t="s">
         <v>35</v>
       </c>
       <c r="T36" s="9">
@@ -3935,7 +4052,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>